<commit_message>
Correct instructions in DS
</commit_message>
<xml_diff>
--- a/longitudinal/dataschema_ProPASS_longitudinal.xlsx
+++ b/longitudinal/dataschema_ProPASS_longitudinal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbtiali\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E80BD47-8912-47EE-AACE-B0BB82368770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25586F3A-128B-4E0A-8312-F4F2C828CD93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2091" uniqueCount="521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2093" uniqueCount="523">
   <si>
     <t>index</t>
   </si>
@@ -1649,6 +1649,12 @@
   </si>
   <si>
     <t>Crosscheck with dis_diabetes_ever.</t>
+  </si>
+  <si>
+    <t>Includes osteoporosis, arthrosis, rheumatic disorder, osteoarthritis or rheumatism, rheumatoid arthritis, osteoarthritis, other arthritis, rheumatoid arthritis.</t>
+  </si>
+  <si>
+    <t>If one or two values are missing from the score, then they can be substituted with the average score of the non-missing items. Questionnaires with more than two missing values should be disregarded.</t>
   </si>
 </sst>
 </file>
@@ -1704,7 +1710,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2021,7 +2027,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F8E0180-A72F-4AF4-960B-1515820225EB}">
   <dimension ref="A1:P113"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.5703125" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
@@ -4924,6 +4930,9 @@
       <c r="L78" t="s">
         <v>46</v>
       </c>
+      <c r="M78" t="s">
+        <v>521</v>
+      </c>
       <c r="N78" t="s">
         <v>323</v>
       </c>
@@ -6156,6 +6165,9 @@
       </c>
       <c r="N111" t="s">
         <v>432</v>
+      </c>
+      <c r="O111" t="s">
+        <v>522</v>
       </c>
     </row>
     <row r="112" spans="1:16" x14ac:dyDescent="0.25">
@@ -6236,7 +6248,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6186D5-BB84-4E3C-AAC4-F17A4EDF9A5A}">
   <dimension ref="A1:F219"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Remove mortality variables from DS
Descision made to harmonize mortality variables separately, so remove from longitudinal DS. Reverts back to V2 of DS.
</commit_message>
<xml_diff>
--- a/longitudinal/dataschema_ProPASS_longitudinal.xlsx
+++ b/longitudinal/dataschema_ProPASS_longitudinal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbtiali\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6511B6D9-5C89-4A28-9051-F7B9BC1EDECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA468C1-B6F0-43C0-AC6A-D201300F230F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2137" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2093" uniqueCount="523">
   <si>
     <t>index</t>
   </si>
@@ -1652,36 +1652,6 @@
   </si>
   <si>
     <t>If one or two values are missing from the score, then they can be substituted with the average score of the non-missing items. Questionnaires with more than two missing values should be disregarded.</t>
-  </si>
-  <si>
-    <t>dth_status</t>
-  </si>
-  <si>
-    <t>Death status</t>
-  </si>
-  <si>
-    <t>Indicator of whether the participant is deceased</t>
-  </si>
-  <si>
-    <t>dth_date_day</t>
-  </si>
-  <si>
-    <t>dth_date_month</t>
-  </si>
-  <si>
-    <t>dth_date_year</t>
-  </si>
-  <si>
-    <t>Death date - Day</t>
-  </si>
-  <si>
-    <t>Death date - Month</t>
-  </si>
-  <si>
-    <t>Death date - Year</t>
-  </si>
-  <si>
-    <t>questionnaire; mortality registry; familly survey</t>
   </si>
   <si>
     <t>propass_fu_3_0</t>
@@ -2056,7 +2026,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F8E0180-A72F-4AF4-960B-1515820225EB}">
-  <dimension ref="A1:P117"/>
+  <dimension ref="A1:P113"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
@@ -2124,7 +2094,7 @@
         <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D2" t="s">
         <v>17</v>
@@ -2153,7 +2123,7 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D3" t="s">
         <v>23</v>
@@ -2182,7 +2152,7 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D4" t="s">
         <v>28</v>
@@ -2211,7 +2181,7 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D5" t="s">
         <v>33</v>
@@ -2243,7 +2213,7 @@
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D6" t="s">
         <v>40</v>
@@ -2284,7 +2254,7 @@
         <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D7" t="s">
         <v>48</v>
@@ -2316,7 +2286,7 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D8" t="s">
         <v>51</v>
@@ -2357,7 +2327,7 @@
         <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D9" t="s">
         <v>57</v>
@@ -2398,7 +2368,7 @@
         <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D10" t="s">
         <v>63</v>
@@ -2439,7 +2409,7 @@
         <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D11" t="s">
         <v>67</v>
@@ -2477,7 +2447,7 @@
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D12" t="s">
         <v>72</v>
@@ -2518,7 +2488,7 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D13" t="s">
         <v>78</v>
@@ -2553,7 +2523,7 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D14" t="s">
         <v>82</v>
@@ -2585,7 +2555,7 @@
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D15" t="s">
         <v>85</v>
@@ -2620,7 +2590,7 @@
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D16" t="s">
         <v>89</v>
@@ -2652,7 +2622,7 @@
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D17" t="s">
         <v>92</v>
@@ -2690,7 +2660,7 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D18" t="s">
         <v>97</v>
@@ -2734,7 +2704,7 @@
         <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D19" t="s">
         <v>105</v>
@@ -2769,7 +2739,7 @@
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D20" t="s">
         <v>108</v>
@@ -2813,7 +2783,7 @@
         <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D21" t="s">
         <v>113</v>
@@ -2848,7 +2818,7 @@
         <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D22" t="s">
         <v>116</v>
@@ -2889,7 +2859,7 @@
         <v>16</v>
       </c>
       <c r="C23" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D23" t="s">
         <v>120</v>
@@ -2933,7 +2903,7 @@
         <v>16</v>
       </c>
       <c r="C24" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D24" t="s">
         <v>124</v>
@@ -2968,7 +2938,7 @@
         <v>16</v>
       </c>
       <c r="C25" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D25" t="s">
         <v>127</v>
@@ -3003,7 +2973,7 @@
         <v>16</v>
       </c>
       <c r="C26" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D26" t="s">
         <v>131</v>
@@ -3035,7 +3005,7 @@
         <v>16</v>
       </c>
       <c r="C27" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D27" t="s">
         <v>133</v>
@@ -3076,7 +3046,7 @@
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D28" t="s">
         <v>139</v>
@@ -3117,7 +3087,7 @@
         <v>16</v>
       </c>
       <c r="C29" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D29" t="s">
         <v>142</v>
@@ -3158,7 +3128,7 @@
         <v>16</v>
       </c>
       <c r="C30" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D30" t="s">
         <v>147</v>
@@ -3199,7 +3169,7 @@
         <v>16</v>
       </c>
       <c r="C31" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D31" t="s">
         <v>152</v>
@@ -3231,7 +3201,7 @@
         <v>16</v>
       </c>
       <c r="C32" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D32" t="s">
         <v>156</v>
@@ -3266,7 +3236,7 @@
         <v>16</v>
       </c>
       <c r="C33" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D33" t="s">
         <v>159</v>
@@ -3301,7 +3271,7 @@
         <v>16</v>
       </c>
       <c r="C34" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D34" t="s">
         <v>162</v>
@@ -3336,7 +3306,7 @@
         <v>16</v>
       </c>
       <c r="C35" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D35" t="s">
         <v>165</v>
@@ -3371,7 +3341,7 @@
         <v>16</v>
       </c>
       <c r="C36" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D36" t="s">
         <v>167</v>
@@ -3406,7 +3376,7 @@
         <v>16</v>
       </c>
       <c r="C37" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D37" t="s">
         <v>169</v>
@@ -3444,7 +3414,7 @@
         <v>16</v>
       </c>
       <c r="C38" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D38" t="s">
         <v>172</v>
@@ -3479,7 +3449,7 @@
         <v>16</v>
       </c>
       <c r="C39" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D39" t="s">
         <v>174</v>
@@ -3514,7 +3484,7 @@
         <v>16</v>
       </c>
       <c r="C40" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D40" t="s">
         <v>177</v>
@@ -3555,7 +3525,7 @@
         <v>16</v>
       </c>
       <c r="C41" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D41" t="s">
         <v>182</v>
@@ -3590,7 +3560,7 @@
         <v>16</v>
       </c>
       <c r="C42" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D42" t="s">
         <v>185</v>
@@ -3631,7 +3601,7 @@
         <v>16</v>
       </c>
       <c r="C43" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D43" t="s">
         <v>189</v>
@@ -3669,7 +3639,7 @@
         <v>16</v>
       </c>
       <c r="C44" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D44" t="s">
         <v>193</v>
@@ -3704,7 +3674,7 @@
         <v>16</v>
       </c>
       <c r="C45" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D45" t="s">
         <v>196</v>
@@ -3748,7 +3718,7 @@
         <v>16</v>
       </c>
       <c r="C46" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D46" t="s">
         <v>202</v>
@@ -3783,7 +3753,7 @@
         <v>16</v>
       </c>
       <c r="C47" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D47" t="s">
         <v>205</v>
@@ -3824,7 +3794,7 @@
         <v>16</v>
       </c>
       <c r="C48" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D48" t="s">
         <v>210</v>
@@ -3862,7 +3832,7 @@
         <v>16</v>
       </c>
       <c r="C49" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D49" t="s">
         <v>213</v>
@@ -3906,7 +3876,7 @@
         <v>16</v>
       </c>
       <c r="C50" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D50" t="s">
         <v>217</v>
@@ -3941,7 +3911,7 @@
         <v>16</v>
       </c>
       <c r="C51" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D51" t="s">
         <v>219</v>
@@ -3976,7 +3946,7 @@
         <v>16</v>
       </c>
       <c r="C52" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D52" t="s">
         <v>222</v>
@@ -4011,7 +3981,7 @@
         <v>16</v>
       </c>
       <c r="C53" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D53" t="s">
         <v>226</v>
@@ -4046,7 +4016,7 @@
         <v>16</v>
       </c>
       <c r="C54" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D54" t="s">
         <v>229</v>
@@ -4078,7 +4048,7 @@
         <v>16</v>
       </c>
       <c r="C55" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D55" t="s">
         <v>231</v>
@@ -4110,7 +4080,7 @@
         <v>16</v>
       </c>
       <c r="C56" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D56" t="s">
         <v>233</v>
@@ -4142,7 +4112,7 @@
         <v>16</v>
       </c>
       <c r="C57" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D57" t="s">
         <v>236</v>
@@ -4177,7 +4147,7 @@
         <v>16</v>
       </c>
       <c r="C58" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D58" t="s">
         <v>239</v>
@@ -4212,7 +4182,7 @@
         <v>16</v>
       </c>
       <c r="C59" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D59" t="s">
         <v>242</v>
@@ -4250,7 +4220,7 @@
         <v>16</v>
       </c>
       <c r="C60" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D60" t="s">
         <v>244</v>
@@ -4282,7 +4252,7 @@
         <v>16</v>
       </c>
       <c r="C61" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D61" t="s">
         <v>247</v>
@@ -4317,7 +4287,7 @@
         <v>16</v>
       </c>
       <c r="C62" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D62" t="s">
         <v>251</v>
@@ -4352,7 +4322,7 @@
         <v>16</v>
       </c>
       <c r="C63" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D63" t="s">
         <v>254</v>
@@ -4390,7 +4360,7 @@
         <v>16</v>
       </c>
       <c r="C64" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D64" t="s">
         <v>258</v>
@@ -4425,7 +4395,7 @@
         <v>16</v>
       </c>
       <c r="C65" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D65" t="s">
         <v>262</v>
@@ -4463,7 +4433,7 @@
         <v>16</v>
       </c>
       <c r="C66" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D66" t="s">
         <v>266</v>
@@ -4498,7 +4468,7 @@
         <v>16</v>
       </c>
       <c r="C67" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D67" t="s">
         <v>270</v>
@@ -4533,7 +4503,7 @@
         <v>16</v>
       </c>
       <c r="C68" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D68" t="s">
         <v>274</v>
@@ -4568,7 +4538,7 @@
         <v>16</v>
       </c>
       <c r="C69" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D69" t="s">
         <v>277</v>
@@ -4609,7 +4579,7 @@
         <v>16</v>
       </c>
       <c r="C70" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D70" t="s">
         <v>283</v>
@@ -4650,7 +4620,7 @@
         <v>16</v>
       </c>
       <c r="C71" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D71" t="s">
         <v>289</v>
@@ -4691,7 +4661,7 @@
         <v>16</v>
       </c>
       <c r="C72" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D72" t="s">
         <v>293</v>
@@ -4732,7 +4702,7 @@
         <v>16</v>
       </c>
       <c r="C73" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D73" t="s">
         <v>297</v>
@@ -4773,7 +4743,7 @@
         <v>16</v>
       </c>
       <c r="C74" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D74" t="s">
         <v>301</v>
@@ -4814,7 +4784,7 @@
         <v>16</v>
       </c>
       <c r="C75" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D75" t="s">
         <v>305</v>
@@ -4855,7 +4825,7 @@
         <v>16</v>
       </c>
       <c r="C76" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D76" t="s">
         <v>309</v>
@@ -4899,7 +4869,7 @@
         <v>16</v>
       </c>
       <c r="C77" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D77" t="s">
         <v>315</v>
@@ -4940,7 +4910,7 @@
         <v>16</v>
       </c>
       <c r="C78" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D78" t="s">
         <v>319</v>
@@ -4978,7 +4948,7 @@
         <v>16</v>
       </c>
       <c r="C79" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D79" t="s">
         <v>323</v>
@@ -5022,7 +4992,7 @@
         <v>16</v>
       </c>
       <c r="C80" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D80" t="s">
         <v>329</v>
@@ -5060,7 +5030,7 @@
         <v>16</v>
       </c>
       <c r="C81" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D81" t="s">
         <v>332</v>
@@ -5101,7 +5071,7 @@
         <v>16</v>
       </c>
       <c r="C82" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D82" t="s">
         <v>338</v>
@@ -5139,7 +5109,7 @@
         <v>16</v>
       </c>
       <c r="C83" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D83" t="s">
         <v>343</v>
@@ -5177,7 +5147,7 @@
         <v>16</v>
       </c>
       <c r="C84" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D84" t="s">
         <v>346</v>
@@ -5215,7 +5185,7 @@
         <v>16</v>
       </c>
       <c r="C85" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D85" t="s">
         <v>350</v>
@@ -5253,7 +5223,7 @@
         <v>16</v>
       </c>
       <c r="C86" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D86" t="s">
         <v>353</v>
@@ -5291,7 +5261,7 @@
         <v>16</v>
       </c>
       <c r="C87" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D87" t="s">
         <v>356</v>
@@ -5329,7 +5299,7 @@
         <v>16</v>
       </c>
       <c r="C88" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D88" t="s">
         <v>359</v>
@@ -5367,7 +5337,7 @@
         <v>16</v>
       </c>
       <c r="C89" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D89" t="s">
         <v>362</v>
@@ -5405,7 +5375,7 @@
         <v>16</v>
       </c>
       <c r="C90" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D90" t="s">
         <v>365</v>
@@ -5443,7 +5413,7 @@
         <v>16</v>
       </c>
       <c r="C91" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D91" t="s">
         <v>368</v>
@@ -5481,7 +5451,7 @@
         <v>16</v>
       </c>
       <c r="C92" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D92" t="s">
         <v>371</v>
@@ -5519,7 +5489,7 @@
         <v>16</v>
       </c>
       <c r="C93" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D93" t="s">
         <v>374</v>
@@ -5557,7 +5527,7 @@
         <v>16</v>
       </c>
       <c r="C94" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D94" t="s">
         <v>377</v>
@@ -5595,7 +5565,7 @@
         <v>16</v>
       </c>
       <c r="C95" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D95" t="s">
         <v>380</v>
@@ -5633,7 +5603,7 @@
         <v>16</v>
       </c>
       <c r="C96" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D96" t="s">
         <v>383</v>
@@ -5671,7 +5641,7 @@
         <v>16</v>
       </c>
       <c r="C97" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D97" t="s">
         <v>386</v>
@@ -5709,7 +5679,7 @@
         <v>16</v>
       </c>
       <c r="C98" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D98" t="s">
         <v>389</v>
@@ -5747,7 +5717,7 @@
         <v>16</v>
       </c>
       <c r="C99" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D99" t="s">
         <v>392</v>
@@ -5785,7 +5755,7 @@
         <v>16</v>
       </c>
       <c r="C100" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D100" t="s">
         <v>395</v>
@@ -5823,7 +5793,7 @@
         <v>16</v>
       </c>
       <c r="C101" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D101" t="s">
         <v>398</v>
@@ -5858,7 +5828,7 @@
         <v>16</v>
       </c>
       <c r="C102" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D102" t="s">
         <v>402</v>
@@ -5893,7 +5863,7 @@
         <v>16</v>
       </c>
       <c r="C103" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D103" t="s">
         <v>406</v>
@@ -5928,7 +5898,7 @@
         <v>16</v>
       </c>
       <c r="C104" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D104" t="s">
         <v>409</v>
@@ -5963,7 +5933,7 @@
         <v>16</v>
       </c>
       <c r="C105" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D105" t="s">
         <v>412</v>
@@ -5998,7 +5968,7 @@
         <v>16</v>
       </c>
       <c r="C106" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D106" t="s">
         <v>415</v>
@@ -6033,7 +6003,7 @@
         <v>16</v>
       </c>
       <c r="C107" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D107" t="s">
         <v>417</v>
@@ -6068,7 +6038,7 @@
         <v>16</v>
       </c>
       <c r="C108" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D108" t="s">
         <v>420</v>
@@ -6103,7 +6073,7 @@
         <v>16</v>
       </c>
       <c r="C109" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D109" t="s">
         <v>423</v>
@@ -6138,7 +6108,7 @@
         <v>16</v>
       </c>
       <c r="C110" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D110" t="s">
         <v>426</v>
@@ -6173,7 +6143,7 @@
         <v>16</v>
       </c>
       <c r="C111" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D111" t="s">
         <v>429</v>
@@ -6211,7 +6181,7 @@
         <v>16</v>
       </c>
       <c r="C112" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D112" t="s">
         <v>432</v>
@@ -6246,7 +6216,7 @@
         <v>16</v>
       </c>
       <c r="C113" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="D113" t="s">
         <v>434</v>
@@ -6271,134 +6241,6 @@
       </c>
       <c r="N113" t="s">
         <v>422</v>
-      </c>
-    </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A114">
-        <v>113</v>
-      </c>
-      <c r="B114" t="s">
-        <v>16</v>
-      </c>
-      <c r="C114" t="s">
-        <v>532</v>
-      </c>
-      <c r="D114" t="s">
-        <v>522</v>
-      </c>
-      <c r="E114" t="s">
-        <v>523</v>
-      </c>
-      <c r="F114" t="s">
-        <v>524</v>
-      </c>
-      <c r="G114" t="s">
-        <v>36</v>
-      </c>
-      <c r="J114" t="s">
-        <v>21</v>
-      </c>
-      <c r="K114" t="s">
-        <v>38</v>
-      </c>
-      <c r="L114" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A115">
-        <v>114</v>
-      </c>
-      <c r="B115" t="s">
-        <v>16</v>
-      </c>
-      <c r="C115" t="s">
-        <v>532</v>
-      </c>
-      <c r="D115" t="s">
-        <v>525</v>
-      </c>
-      <c r="E115" t="s">
-        <v>528</v>
-      </c>
-      <c r="F115" t="s">
-        <v>528</v>
-      </c>
-      <c r="G115" t="s">
-        <v>36</v>
-      </c>
-      <c r="J115" t="s">
-        <v>21</v>
-      </c>
-      <c r="K115" t="s">
-        <v>38</v>
-      </c>
-      <c r="L115" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A116">
-        <v>115</v>
-      </c>
-      <c r="B116" t="s">
-        <v>16</v>
-      </c>
-      <c r="C116" t="s">
-        <v>532</v>
-      </c>
-      <c r="D116" t="s">
-        <v>526</v>
-      </c>
-      <c r="E116" t="s">
-        <v>529</v>
-      </c>
-      <c r="F116" t="s">
-        <v>529</v>
-      </c>
-      <c r="G116" t="s">
-        <v>36</v>
-      </c>
-      <c r="J116" t="s">
-        <v>21</v>
-      </c>
-      <c r="K116" t="s">
-        <v>38</v>
-      </c>
-      <c r="L116" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A117">
-        <v>116</v>
-      </c>
-      <c r="B117" t="s">
-        <v>16</v>
-      </c>
-      <c r="C117" t="s">
-        <v>532</v>
-      </c>
-      <c r="D117" t="s">
-        <v>527</v>
-      </c>
-      <c r="E117" t="s">
-        <v>530</v>
-      </c>
-      <c r="F117" t="s">
-        <v>530</v>
-      </c>
-      <c r="G117" t="s">
-        <v>36</v>
-      </c>
-      <c r="J117" t="s">
-        <v>21</v>
-      </c>
-      <c r="K117" t="s">
-        <v>38</v>
-      </c>
-      <c r="L117" t="s">
-        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -6408,7 +6250,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6186D5-BB84-4E3C-AAC4-F17A4EDF9A5A}">
-  <dimension ref="A1:F221"/>
+  <dimension ref="A1:F219"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
@@ -6444,7 +6286,7 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C2" t="s">
         <v>48</v>
@@ -6464,7 +6306,7 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
@@ -6484,7 +6326,7 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C4" t="s">
         <v>57</v>
@@ -6504,7 +6346,7 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C5" t="s">
         <v>57</v>
@@ -6524,7 +6366,7 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C6" t="s">
         <v>57</v>
@@ -6544,7 +6386,7 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C7" t="s">
         <v>57</v>
@@ -6564,7 +6406,7 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C8" t="s">
         <v>63</v>
@@ -6584,7 +6426,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C9" t="s">
         <v>63</v>
@@ -6604,7 +6446,7 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C10" t="s">
         <v>67</v>
@@ -6624,7 +6466,7 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C11" t="s">
         <v>67</v>
@@ -6644,7 +6486,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C12" t="s">
         <v>72</v>
@@ -6664,7 +6506,7 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C13" t="s">
         <v>72</v>
@@ -6684,7 +6526,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C14" t="s">
         <v>85</v>
@@ -6704,7 +6546,7 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C15" t="s">
         <v>85</v>
@@ -6724,7 +6566,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C16" t="s">
         <v>89</v>
@@ -6744,7 +6586,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C17" t="s">
         <v>89</v>
@@ -6764,7 +6606,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C18" t="s">
         <v>89</v>
@@ -6784,7 +6626,7 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C19" t="s">
         <v>89</v>
@@ -6804,7 +6646,7 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C20" t="s">
         <v>92</v>
@@ -6824,7 +6666,7 @@
         <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C21" t="s">
         <v>92</v>
@@ -6844,7 +6686,7 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C22" t="s">
         <v>105</v>
@@ -6864,7 +6706,7 @@
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C23" t="s">
         <v>105</v>
@@ -6884,7 +6726,7 @@
         <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C24" t="s">
         <v>113</v>
@@ -6904,7 +6746,7 @@
         <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C25" t="s">
         <v>113</v>
@@ -6924,7 +6766,7 @@
         <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C26" t="s">
         <v>124</v>
@@ -6944,7 +6786,7 @@
         <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C27" t="s">
         <v>124</v>
@@ -6964,7 +6806,7 @@
         <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C28" t="s">
         <v>152</v>
@@ -6984,7 +6826,7 @@
         <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C29" t="s">
         <v>152</v>
@@ -7004,7 +6846,7 @@
         <v>16</v>
       </c>
       <c r="B30" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C30" t="s">
         <v>152</v>
@@ -7024,7 +6866,7 @@
         <v>16</v>
       </c>
       <c r="B31" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C31" t="s">
         <v>182</v>
@@ -7044,7 +6886,7 @@
         <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C32" t="s">
         <v>182</v>
@@ -7064,7 +6906,7 @@
         <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C33" t="s">
         <v>182</v>
@@ -7084,7 +6926,7 @@
         <v>16</v>
       </c>
       <c r="B34" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C34" t="s">
         <v>189</v>
@@ -7104,7 +6946,7 @@
         <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C35" t="s">
         <v>189</v>
@@ -7124,7 +6966,7 @@
         <v>16</v>
       </c>
       <c r="B36" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C36" t="s">
         <v>189</v>
@@ -7144,7 +6986,7 @@
         <v>16</v>
       </c>
       <c r="B37" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C37" t="s">
         <v>202</v>
@@ -7164,7 +7006,7 @@
         <v>16</v>
       </c>
       <c r="B38" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C38" t="s">
         <v>202</v>
@@ -7184,7 +7026,7 @@
         <v>16</v>
       </c>
       <c r="B39" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C39" t="s">
         <v>202</v>
@@ -7204,7 +7046,7 @@
         <v>16</v>
       </c>
       <c r="B40" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C40" t="s">
         <v>202</v>
@@ -7224,7 +7066,7 @@
         <v>16</v>
       </c>
       <c r="B41" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C41" t="s">
         <v>205</v>
@@ -7244,7 +7086,7 @@
         <v>16</v>
       </c>
       <c r="B42" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C42" t="s">
         <v>205</v>
@@ -7264,7 +7106,7 @@
         <v>16</v>
       </c>
       <c r="B43" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C43" t="s">
         <v>205</v>
@@ -7284,7 +7126,7 @@
         <v>16</v>
       </c>
       <c r="B44" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C44" t="s">
         <v>210</v>
@@ -7304,7 +7146,7 @@
         <v>16</v>
       </c>
       <c r="B45" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C45" t="s">
         <v>210</v>
@@ -7324,7 +7166,7 @@
         <v>16</v>
       </c>
       <c r="B46" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C46" t="s">
         <v>219</v>
@@ -7344,7 +7186,7 @@
         <v>16</v>
       </c>
       <c r="B47" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C47" t="s">
         <v>219</v>
@@ -7364,7 +7206,7 @@
         <v>16</v>
       </c>
       <c r="B48" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C48" t="s">
         <v>219</v>
@@ -7384,7 +7226,7 @@
         <v>16</v>
       </c>
       <c r="B49" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C49" t="s">
         <v>219</v>
@@ -7404,7 +7246,7 @@
         <v>16</v>
       </c>
       <c r="B50" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C50" t="s">
         <v>219</v>
@@ -7424,7 +7266,7 @@
         <v>16</v>
       </c>
       <c r="B51" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C51" t="s">
         <v>219</v>
@@ -7444,7 +7286,7 @@
         <v>16</v>
       </c>
       <c r="B52" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C52" t="s">
         <v>219</v>
@@ -7464,7 +7306,7 @@
         <v>16</v>
       </c>
       <c r="B53" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C53" t="s">
         <v>219</v>
@@ -7484,7 +7326,7 @@
         <v>16</v>
       </c>
       <c r="B54" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C54" t="s">
         <v>219</v>
@@ -7504,7 +7346,7 @@
         <v>16</v>
       </c>
       <c r="B55" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C55" t="s">
         <v>222</v>
@@ -7524,7 +7366,7 @@
         <v>16</v>
       </c>
       <c r="B56" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C56" t="s">
         <v>222</v>
@@ -7544,7 +7386,7 @@
         <v>16</v>
       </c>
       <c r="B57" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C57" t="s">
         <v>226</v>
@@ -7564,7 +7406,7 @@
         <v>16</v>
       </c>
       <c r="B58" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C58" t="s">
         <v>226</v>
@@ -7584,7 +7426,7 @@
         <v>16</v>
       </c>
       <c r="B59" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C59" t="s">
         <v>226</v>
@@ -7604,7 +7446,7 @@
         <v>16</v>
       </c>
       <c r="B60" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C60" t="s">
         <v>229</v>
@@ -7624,7 +7466,7 @@
         <v>16</v>
       </c>
       <c r="B61" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C61" t="s">
         <v>229</v>
@@ -7644,7 +7486,7 @@
         <v>16</v>
       </c>
       <c r="B62" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C62" t="s">
         <v>229</v>
@@ -7664,7 +7506,7 @@
         <v>16</v>
       </c>
       <c r="B63" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C63" t="s">
         <v>231</v>
@@ -7684,7 +7526,7 @@
         <v>16</v>
       </c>
       <c r="B64" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C64" t="s">
         <v>231</v>
@@ -7704,7 +7546,7 @@
         <v>16</v>
       </c>
       <c r="B65" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C65" t="s">
         <v>231</v>
@@ -7724,7 +7566,7 @@
         <v>16</v>
       </c>
       <c r="B66" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C66" t="s">
         <v>233</v>
@@ -7744,7 +7586,7 @@
         <v>16</v>
       </c>
       <c r="B67" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C67" t="s">
         <v>233</v>
@@ -7764,7 +7606,7 @@
         <v>16</v>
       </c>
       <c r="B68" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C68" t="s">
         <v>233</v>
@@ -7784,7 +7626,7 @@
         <v>16</v>
       </c>
       <c r="B69" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C69" t="s">
         <v>233</v>
@@ -7804,7 +7646,7 @@
         <v>16</v>
       </c>
       <c r="B70" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C70" t="s">
         <v>233</v>
@@ -7824,7 +7666,7 @@
         <v>16</v>
       </c>
       <c r="B71" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C71" t="s">
         <v>233</v>
@@ -7844,7 +7686,7 @@
         <v>16</v>
       </c>
       <c r="B72" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C72" t="s">
         <v>233</v>
@@ -7864,7 +7706,7 @@
         <v>16</v>
       </c>
       <c r="B73" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C73" t="s">
         <v>233</v>
@@ -7884,7 +7726,7 @@
         <v>16</v>
       </c>
       <c r="B74" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C74" t="s">
         <v>233</v>
@@ -7904,7 +7746,7 @@
         <v>16</v>
       </c>
       <c r="B75" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C75" t="s">
         <v>233</v>
@@ -7924,7 +7766,7 @@
         <v>16</v>
       </c>
       <c r="B76" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C76" t="s">
         <v>233</v>
@@ -7944,7 +7786,7 @@
         <v>16</v>
       </c>
       <c r="B77" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C77" t="s">
         <v>236</v>
@@ -7964,7 +7806,7 @@
         <v>16</v>
       </c>
       <c r="B78" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C78" t="s">
         <v>236</v>
@@ -7984,7 +7826,7 @@
         <v>16</v>
       </c>
       <c r="B79" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C79" t="s">
         <v>236</v>
@@ -8004,7 +7846,7 @@
         <v>16</v>
       </c>
       <c r="B80" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C80" t="s">
         <v>239</v>
@@ -8024,7 +7866,7 @@
         <v>16</v>
       </c>
       <c r="B81" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C81" t="s">
         <v>239</v>
@@ -8044,7 +7886,7 @@
         <v>16</v>
       </c>
       <c r="B82" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C82" t="s">
         <v>239</v>
@@ -8064,7 +7906,7 @@
         <v>16</v>
       </c>
       <c r="B83" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C83" t="s">
         <v>244</v>
@@ -8084,7 +7926,7 @@
         <v>16</v>
       </c>
       <c r="B84" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C84" t="s">
         <v>244</v>
@@ -8104,7 +7946,7 @@
         <v>16</v>
       </c>
       <c r="B85" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C85" t="s">
         <v>244</v>
@@ -8124,7 +7966,7 @@
         <v>16</v>
       </c>
       <c r="B86" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C86" t="s">
         <v>244</v>
@@ -8144,7 +7986,7 @@
         <v>16</v>
       </c>
       <c r="B87" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C87" t="s">
         <v>244</v>
@@ -8164,7 +8006,7 @@
         <v>16</v>
       </c>
       <c r="B88" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C88" t="s">
         <v>244</v>
@@ -8184,7 +8026,7 @@
         <v>16</v>
       </c>
       <c r="B89" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C89" t="s">
         <v>247</v>
@@ -8204,7 +8046,7 @@
         <v>16</v>
       </c>
       <c r="B90" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C90" t="s">
         <v>247</v>
@@ -8224,7 +8066,7 @@
         <v>16</v>
       </c>
       <c r="B91" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C91" t="s">
         <v>247</v>
@@ -8244,7 +8086,7 @@
         <v>16</v>
       </c>
       <c r="B92" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C92" t="s">
         <v>251</v>
@@ -8264,7 +8106,7 @@
         <v>16</v>
       </c>
       <c r="B93" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C93" t="s">
         <v>251</v>
@@ -8284,7 +8126,7 @@
         <v>16</v>
       </c>
       <c r="B94" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C94" t="s">
         <v>251</v>
@@ -8304,7 +8146,7 @@
         <v>16</v>
       </c>
       <c r="B95" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C95" t="s">
         <v>251</v>
@@ -8324,7 +8166,7 @@
         <v>16</v>
       </c>
       <c r="B96" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C96" t="s">
         <v>254</v>
@@ -8344,7 +8186,7 @@
         <v>16</v>
       </c>
       <c r="B97" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C97" t="s">
         <v>254</v>
@@ -8364,7 +8206,7 @@
         <v>16</v>
       </c>
       <c r="B98" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C98" t="s">
         <v>258</v>
@@ -8384,7 +8226,7 @@
         <v>16</v>
       </c>
       <c r="B99" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C99" t="s">
         <v>258</v>
@@ -8404,7 +8246,7 @@
         <v>16</v>
       </c>
       <c r="B100" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C100" t="s">
         <v>262</v>
@@ -8424,7 +8266,7 @@
         <v>16</v>
       </c>
       <c r="B101" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C101" t="s">
         <v>262</v>
@@ -8444,7 +8286,7 @@
         <v>16</v>
       </c>
       <c r="B102" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C102" t="s">
         <v>274</v>
@@ -8464,7 +8306,7 @@
         <v>16</v>
       </c>
       <c r="B103" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C103" t="s">
         <v>274</v>
@@ -8484,7 +8326,7 @@
         <v>16</v>
       </c>
       <c r="B104" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C104" t="s">
         <v>274</v>
@@ -8504,7 +8346,7 @@
         <v>16</v>
       </c>
       <c r="B105" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C105" t="s">
         <v>274</v>
@@ -8524,7 +8366,7 @@
         <v>16</v>
       </c>
       <c r="B106" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C106" t="s">
         <v>277</v>
@@ -8544,7 +8386,7 @@
         <v>16</v>
       </c>
       <c r="B107" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C107" t="s">
         <v>277</v>
@@ -8564,7 +8406,7 @@
         <v>16</v>
       </c>
       <c r="B108" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C108" t="s">
         <v>277</v>
@@ -8584,7 +8426,7 @@
         <v>16</v>
       </c>
       <c r="B109" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C109" t="s">
         <v>283</v>
@@ -8604,7 +8446,7 @@
         <v>16</v>
       </c>
       <c r="B110" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C110" t="s">
         <v>283</v>
@@ -8624,7 +8466,7 @@
         <v>16</v>
       </c>
       <c r="B111" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C111" t="s">
         <v>283</v>
@@ -8644,7 +8486,7 @@
         <v>16</v>
       </c>
       <c r="B112" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C112" t="s">
         <v>289</v>
@@ -8664,7 +8506,7 @@
         <v>16</v>
       </c>
       <c r="B113" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C113" t="s">
         <v>289</v>
@@ -8684,7 +8526,7 @@
         <v>16</v>
       </c>
       <c r="B114" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C114" t="s">
         <v>289</v>
@@ -8704,7 +8546,7 @@
         <v>16</v>
       </c>
       <c r="B115" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C115" t="s">
         <v>293</v>
@@ -8724,7 +8566,7 @@
         <v>16</v>
       </c>
       <c r="B116" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C116" t="s">
         <v>293</v>
@@ -8744,7 +8586,7 @@
         <v>16</v>
       </c>
       <c r="B117" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C117" t="s">
         <v>293</v>
@@ -8764,7 +8606,7 @@
         <v>16</v>
       </c>
       <c r="B118" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C118" t="s">
         <v>297</v>
@@ -8784,7 +8626,7 @@
         <v>16</v>
       </c>
       <c r="B119" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C119" t="s">
         <v>297</v>
@@ -8804,7 +8646,7 @@
         <v>16</v>
       </c>
       <c r="B120" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C120" t="s">
         <v>297</v>
@@ -8824,7 +8666,7 @@
         <v>16</v>
       </c>
       <c r="B121" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C121" t="s">
         <v>301</v>
@@ -8844,7 +8686,7 @@
         <v>16</v>
       </c>
       <c r="B122" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C122" t="s">
         <v>301</v>
@@ -8864,7 +8706,7 @@
         <v>16</v>
       </c>
       <c r="B123" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C123" t="s">
         <v>301</v>
@@ -8884,7 +8726,7 @@
         <v>16</v>
       </c>
       <c r="B124" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C124" t="s">
         <v>305</v>
@@ -8904,7 +8746,7 @@
         <v>16</v>
       </c>
       <c r="B125" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C125" t="s">
         <v>305</v>
@@ -8924,7 +8766,7 @@
         <v>16</v>
       </c>
       <c r="B126" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C126" t="s">
         <v>305</v>
@@ -8944,7 +8786,7 @@
         <v>16</v>
       </c>
       <c r="B127" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C127" t="s">
         <v>309</v>
@@ -8964,7 +8806,7 @@
         <v>16</v>
       </c>
       <c r="B128" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C128" t="s">
         <v>309</v>
@@ -8984,7 +8826,7 @@
         <v>16</v>
       </c>
       <c r="B129" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C129" t="s">
         <v>309</v>
@@ -9004,7 +8846,7 @@
         <v>16</v>
       </c>
       <c r="B130" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C130" t="s">
         <v>315</v>
@@ -9024,7 +8866,7 @@
         <v>16</v>
       </c>
       <c r="B131" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C131" t="s">
         <v>315</v>
@@ -9044,7 +8886,7 @@
         <v>16</v>
       </c>
       <c r="B132" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C132" t="s">
         <v>315</v>
@@ -9064,7 +8906,7 @@
         <v>16</v>
       </c>
       <c r="B133" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C133" t="s">
         <v>319</v>
@@ -9084,7 +8926,7 @@
         <v>16</v>
       </c>
       <c r="B134" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C134" t="s">
         <v>319</v>
@@ -9104,7 +8946,7 @@
         <v>16</v>
       </c>
       <c r="B135" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C135" t="s">
         <v>319</v>
@@ -9124,7 +8966,7 @@
         <v>16</v>
       </c>
       <c r="B136" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C136" t="s">
         <v>323</v>
@@ -9144,7 +8986,7 @@
         <v>16</v>
       </c>
       <c r="B137" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C137" t="s">
         <v>323</v>
@@ -9164,7 +9006,7 @@
         <v>16</v>
       </c>
       <c r="B138" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C138" t="s">
         <v>323</v>
@@ -9184,7 +9026,7 @@
         <v>16</v>
       </c>
       <c r="B139" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C139" t="s">
         <v>329</v>
@@ -9204,7 +9046,7 @@
         <v>16</v>
       </c>
       <c r="B140" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C140" t="s">
         <v>329</v>
@@ -9224,7 +9066,7 @@
         <v>16</v>
       </c>
       <c r="B141" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C141" t="s">
         <v>329</v>
@@ -9244,7 +9086,7 @@
         <v>16</v>
       </c>
       <c r="B142" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C142" t="s">
         <v>332</v>
@@ -9264,7 +9106,7 @@
         <v>16</v>
       </c>
       <c r="B143" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C143" t="s">
         <v>332</v>
@@ -9284,7 +9126,7 @@
         <v>16</v>
       </c>
       <c r="B144" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C144" t="s">
         <v>332</v>
@@ -9304,7 +9146,7 @@
         <v>16</v>
       </c>
       <c r="B145" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C145" t="s">
         <v>338</v>
@@ -9324,7 +9166,7 @@
         <v>16</v>
       </c>
       <c r="B146" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C146" t="s">
         <v>338</v>
@@ -9344,7 +9186,7 @@
         <v>16</v>
       </c>
       <c r="B147" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C147" t="s">
         <v>338</v>
@@ -9364,7 +9206,7 @@
         <v>16</v>
       </c>
       <c r="B148" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C148" t="s">
         <v>343</v>
@@ -9384,7 +9226,7 @@
         <v>16</v>
       </c>
       <c r="B149" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C149" t="s">
         <v>343</v>
@@ -9404,7 +9246,7 @@
         <v>16</v>
       </c>
       <c r="B150" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C150" t="s">
         <v>343</v>
@@ -9424,7 +9266,7 @@
         <v>16</v>
       </c>
       <c r="B151" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C151" t="s">
         <v>346</v>
@@ -9444,7 +9286,7 @@
         <v>16</v>
       </c>
       <c r="B152" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C152" t="s">
         <v>346</v>
@@ -9464,7 +9306,7 @@
         <v>16</v>
       </c>
       <c r="B153" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C153" t="s">
         <v>346</v>
@@ -9484,7 +9326,7 @@
         <v>16</v>
       </c>
       <c r="B154" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C154" t="s">
         <v>350</v>
@@ -9504,7 +9346,7 @@
         <v>16</v>
       </c>
       <c r="B155" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C155" t="s">
         <v>350</v>
@@ -9524,7 +9366,7 @@
         <v>16</v>
       </c>
       <c r="B156" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C156" t="s">
         <v>350</v>
@@ -9544,7 +9386,7 @@
         <v>16</v>
       </c>
       <c r="B157" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C157" t="s">
         <v>353</v>
@@ -9564,7 +9406,7 @@
         <v>16</v>
       </c>
       <c r="B158" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C158" t="s">
         <v>353</v>
@@ -9584,7 +9426,7 @@
         <v>16</v>
       </c>
       <c r="B159" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C159" t="s">
         <v>353</v>
@@ -9604,7 +9446,7 @@
         <v>16</v>
       </c>
       <c r="B160" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C160" t="s">
         <v>356</v>
@@ -9624,7 +9466,7 @@
         <v>16</v>
       </c>
       <c r="B161" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C161" t="s">
         <v>356</v>
@@ -9644,7 +9486,7 @@
         <v>16</v>
       </c>
       <c r="B162" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C162" t="s">
         <v>356</v>
@@ -9664,7 +9506,7 @@
         <v>16</v>
       </c>
       <c r="B163" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C163" t="s">
         <v>359</v>
@@ -9684,7 +9526,7 @@
         <v>16</v>
       </c>
       <c r="B164" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C164" t="s">
         <v>359</v>
@@ -9704,7 +9546,7 @@
         <v>16</v>
       </c>
       <c r="B165" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C165" t="s">
         <v>359</v>
@@ -9724,7 +9566,7 @@
         <v>16</v>
       </c>
       <c r="B166" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C166" t="s">
         <v>362</v>
@@ -9744,7 +9586,7 @@
         <v>16</v>
       </c>
       <c r="B167" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C167" t="s">
         <v>362</v>
@@ -9764,7 +9606,7 @@
         <v>16</v>
       </c>
       <c r="B168" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C168" t="s">
         <v>362</v>
@@ -9784,7 +9626,7 @@
         <v>16</v>
       </c>
       <c r="B169" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C169" t="s">
         <v>365</v>
@@ -9804,7 +9646,7 @@
         <v>16</v>
       </c>
       <c r="B170" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C170" t="s">
         <v>365</v>
@@ -9824,7 +9666,7 @@
         <v>16</v>
       </c>
       <c r="B171" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C171" t="s">
         <v>365</v>
@@ -9844,7 +9686,7 @@
         <v>16</v>
       </c>
       <c r="B172" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C172" t="s">
         <v>368</v>
@@ -9864,7 +9706,7 @@
         <v>16</v>
       </c>
       <c r="B173" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C173" t="s">
         <v>368</v>
@@ -9884,7 +9726,7 @@
         <v>16</v>
       </c>
       <c r="B174" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C174" t="s">
         <v>368</v>
@@ -9904,7 +9746,7 @@
         <v>16</v>
       </c>
       <c r="B175" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C175" t="s">
         <v>371</v>
@@ -9924,7 +9766,7 @@
         <v>16</v>
       </c>
       <c r="B176" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C176" t="s">
         <v>371</v>
@@ -9944,7 +9786,7 @@
         <v>16</v>
       </c>
       <c r="B177" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C177" t="s">
         <v>371</v>
@@ -9964,7 +9806,7 @@
         <v>16</v>
       </c>
       <c r="B178" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C178" t="s">
         <v>374</v>
@@ -9984,7 +9826,7 @@
         <v>16</v>
       </c>
       <c r="B179" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C179" t="s">
         <v>374</v>
@@ -10004,7 +9846,7 @@
         <v>16</v>
       </c>
       <c r="B180" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C180" t="s">
         <v>374</v>
@@ -10024,7 +9866,7 @@
         <v>16</v>
       </c>
       <c r="B181" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C181" t="s">
         <v>377</v>
@@ -10044,7 +9886,7 @@
         <v>16</v>
       </c>
       <c r="B182" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C182" t="s">
         <v>377</v>
@@ -10064,7 +9906,7 @@
         <v>16</v>
       </c>
       <c r="B183" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C183" t="s">
         <v>377</v>
@@ -10084,7 +9926,7 @@
         <v>16</v>
       </c>
       <c r="B184" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C184" t="s">
         <v>380</v>
@@ -10104,7 +9946,7 @@
         <v>16</v>
       </c>
       <c r="B185" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C185" t="s">
         <v>380</v>
@@ -10124,7 +9966,7 @@
         <v>16</v>
       </c>
       <c r="B186" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C186" t="s">
         <v>380</v>
@@ -10144,7 +9986,7 @@
         <v>16</v>
       </c>
       <c r="B187" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C187" t="s">
         <v>383</v>
@@ -10164,7 +10006,7 @@
         <v>16</v>
       </c>
       <c r="B188" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C188" t="s">
         <v>383</v>
@@ -10184,7 +10026,7 @@
         <v>16</v>
       </c>
       <c r="B189" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C189" t="s">
         <v>383</v>
@@ -10204,7 +10046,7 @@
         <v>16</v>
       </c>
       <c r="B190" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C190" t="s">
         <v>386</v>
@@ -10224,7 +10066,7 @@
         <v>16</v>
       </c>
       <c r="B191" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C191" t="s">
         <v>386</v>
@@ -10244,7 +10086,7 @@
         <v>16</v>
       </c>
       <c r="B192" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C192" t="s">
         <v>386</v>
@@ -10264,7 +10106,7 @@
         <v>16</v>
       </c>
       <c r="B193" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C193" t="s">
         <v>389</v>
@@ -10284,7 +10126,7 @@
         <v>16</v>
       </c>
       <c r="B194" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C194" t="s">
         <v>389</v>
@@ -10304,7 +10146,7 @@
         <v>16</v>
       </c>
       <c r="B195" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C195" t="s">
         <v>389</v>
@@ -10324,7 +10166,7 @@
         <v>16</v>
       </c>
       <c r="B196" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C196" t="s">
         <v>392</v>
@@ -10344,7 +10186,7 @@
         <v>16</v>
       </c>
       <c r="B197" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C197" t="s">
         <v>392</v>
@@ -10364,7 +10206,7 @@
         <v>16</v>
       </c>
       <c r="B198" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C198" t="s">
         <v>392</v>
@@ -10384,7 +10226,7 @@
         <v>16</v>
       </c>
       <c r="B199" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C199" t="s">
         <v>395</v>
@@ -10404,7 +10246,7 @@
         <v>16</v>
       </c>
       <c r="B200" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C200" t="s">
         <v>395</v>
@@ -10424,7 +10266,7 @@
         <v>16</v>
       </c>
       <c r="B201" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C201" t="s">
         <v>395</v>
@@ -10444,7 +10286,7 @@
         <v>16</v>
       </c>
       <c r="B202" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C202" t="s">
         <v>398</v>
@@ -10464,7 +10306,7 @@
         <v>16</v>
       </c>
       <c r="B203" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C203" t="s">
         <v>398</v>
@@ -10484,7 +10326,7 @@
         <v>16</v>
       </c>
       <c r="B204" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C204" t="s">
         <v>398</v>
@@ -10504,7 +10346,7 @@
         <v>16</v>
       </c>
       <c r="B205" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C205" t="s">
         <v>402</v>
@@ -10524,7 +10366,7 @@
         <v>16</v>
       </c>
       <c r="B206" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C206" t="s">
         <v>402</v>
@@ -10544,7 +10386,7 @@
         <v>16</v>
       </c>
       <c r="B207" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C207" t="s">
         <v>402</v>
@@ -10564,7 +10406,7 @@
         <v>16</v>
       </c>
       <c r="B208" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C208" t="s">
         <v>406</v>
@@ -10584,7 +10426,7 @@
         <v>16</v>
       </c>
       <c r="B209" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C209" t="s">
         <v>406</v>
@@ -10604,7 +10446,7 @@
         <v>16</v>
       </c>
       <c r="B210" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C210" t="s">
         <v>406</v>
@@ -10624,7 +10466,7 @@
         <v>16</v>
       </c>
       <c r="B211" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C211" t="s">
         <v>409</v>
@@ -10644,7 +10486,7 @@
         <v>16</v>
       </c>
       <c r="B212" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C212" t="s">
         <v>409</v>
@@ -10664,7 +10506,7 @@
         <v>16</v>
       </c>
       <c r="B213" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C213" t="s">
         <v>409</v>
@@ -10684,7 +10526,7 @@
         <v>16</v>
       </c>
       <c r="B214" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C214" t="s">
         <v>412</v>
@@ -10704,7 +10546,7 @@
         <v>16</v>
       </c>
       <c r="B215" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C215" t="s">
         <v>412</v>
@@ -10724,7 +10566,7 @@
         <v>16</v>
       </c>
       <c r="B216" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C216" t="s">
         <v>412</v>
@@ -10744,7 +10586,7 @@
         <v>16</v>
       </c>
       <c r="B217" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C217" t="s">
         <v>415</v>
@@ -10764,7 +10606,7 @@
         <v>16</v>
       </c>
       <c r="B218" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C218" t="s">
         <v>415</v>
@@ -10784,7 +10626,7 @@
         <v>16</v>
       </c>
       <c r="B219" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="C219" t="s">
         <v>415</v>
@@ -10797,46 +10639,6 @@
       </c>
       <c r="F219" t="s">
         <v>515</v>
-      </c>
-    </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A220" t="s">
-        <v>16</v>
-      </c>
-      <c r="B220" t="s">
-        <v>532</v>
-      </c>
-      <c r="C220" t="s">
-        <v>522</v>
-      </c>
-      <c r="D220">
-        <v>0</v>
-      </c>
-      <c r="E220">
-        <v>0</v>
-      </c>
-      <c r="F220" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A221" t="s">
-        <v>16</v>
-      </c>
-      <c r="B221" t="s">
-        <v>532</v>
-      </c>
-      <c r="C221" t="s">
-        <v>522</v>
-      </c>
-      <c r="D221">
-        <v>0</v>
-      </c>
-      <c r="E221">
-        <v>1</v>
-      </c>
-      <c r="F221" t="s">
-        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change table name to 2_0
</commit_message>
<xml_diff>
--- a/longitudinal/dataschema_ProPASS_longitudinal.xlsx
+++ b/longitudinal/dataschema_ProPASS_longitudinal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA468C1-B6F0-43C0-AC6A-D201300F230F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F151F5-988E-48DA-A998-6D73ACFF3F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
+    <workbookView xWindow="19090" yWindow="1840" windowWidth="19420" windowHeight="10300" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -1654,17 +1654,23 @@
     <t>If one or two values are missing from the score, then they can be substituted with the average score of the non-missing items. Questionnaires with more than two missing values should be disregarded.</t>
   </si>
   <si>
-    <t>propass_fu_3_0</t>
+    <t>propass_fu_2_0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -6244,6 +6250,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -10642,6 +10649,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>